<commit_message>
update: Hyatt Place Busan Yeonsan Trip.com score to 8.8 and reviews to 63
</commit_message>
<xml_diff>
--- a/韓國釜山2026年12月住宿評比與比價總表.xlsx
+++ b/韓國釜山2026年12月住宿評比與比價總表.xlsx
@@ -6190,7 +6190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F139"/>
+  <dimension ref="A1:F140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="49" customWidth="1" min="1" max="1"/>
@@ -10626,6 +10626,38 @@
       <c r="F139" s="5" t="inlineStr">
         <is>
           <t>KTX Busan Station Near International Coffee Museum</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="20" customHeight="1">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>Hyatt Place Busan Yeonsan</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>4星級</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>TWD 4,360 / 晚 (總額 TWD 23,980)</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>8.8</t>
+        </is>
+      </c>
+      <c r="E140" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Yeonsan Near Yeonsan Metro Station</t>
         </is>
       </c>
     </row>
@@ -24317,9 +24349,9 @@
           <t>8.7 (17 則評價)</t>
         </is>
       </c>
-      <c r="E61" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="E61" s="15" t="inlineStr">
+        <is>
+          <t>8.8 (63 則評價)</t>
         </is>
       </c>
       <c r="F61" s="15" t="inlineStr">
@@ -24344,12 +24376,12 @@
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>TWD 4,360 / 晚 (總額 TWD 23,980)</t>
         </is>
       </c>
       <c r="K61" s="14" t="inlineStr">
         <is>
-          <t>8.77 / 10 (597.0 則總評價)</t>
+          <t>8.77 / 10 (660.0 則總評價)</t>
         </is>
       </c>
     </row>

</xml_diff>